<commit_message>
Code using standard variables
</commit_message>
<xml_diff>
--- a/provider_specialty_cprd_V.0.4.xlsx
+++ b/provider_specialty_cprd_V.0.4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioxfordnexus-my.sharepoint.com/personal/orms0952_ox_ac_uk/Documents/OMOP_Validation study/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{03CD51DF-2ED6-4E6D-9395-4CAD2A3CE9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A581B4A-EB61-4D59-A745-6984BACAC491}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{03CD51DF-2ED6-4E6D-9395-4CAD2A3CE9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B198807-D701-4EAC-AD25-C244C2969FF4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{46870897-BCFD-414C-A471-BD3159C3E0A3}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$63</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="117">
   <si>
     <t>specialty_concept_id</t>
   </si>
@@ -50,9 +50,6 @@
     <t>specialty_source_value</t>
   </si>
   <si>
-    <t>Include</t>
-  </si>
-  <si>
     <t>unit_cost</t>
   </si>
   <si>
@@ -387,6 +384,12 @@
   </si>
   <si>
     <t>Associate Practitioner - General Practitioner</t>
+  </si>
+  <si>
+    <t>Include_source</t>
+  </si>
+  <si>
+    <t>Include_standard</t>
   </si>
 </sst>
 </file>
@@ -770,17 +773,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01908DF-AC8E-4A47-8381-A0A0F45C789A}">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="61" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" customWidth="1"/>
-    <col min="7" max="7" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="255.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -791,1275 +797,1464 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>38004185</v>
       </c>
       <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
       <c r="D2">
         <v>0</v>
       </c>
-      <c r="E2" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>38003696</v>
       </c>
       <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="G3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2">
-        <v>23.5</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>10</v>
       </c>
-      <c r="G3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>38004185</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
-      <c r="E4" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>38004154</v>
       </c>
       <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>38003627</v>
       </c>
       <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2">
+        <v>41</v>
+      </c>
+      <c r="G6" t="s">
         <v>16</v>
       </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" s="2">
-        <v>41</v>
-      </c>
-      <c r="F6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>38003810</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
-      <c r="E7" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>38003648</v>
       </c>
       <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
         <v>19</v>
       </c>
-      <c r="C8" t="s">
-        <v>20</v>
-      </c>
       <c r="D8">
         <v>0</v>
       </c>
-      <c r="E8" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>38003789</v>
       </c>
       <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
         <v>21</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2">
+        <v>31.72</v>
+      </c>
+      <c r="G9" t="s">
         <v>22</v>
       </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9" s="2">
-        <v>31.72</v>
-      </c>
-      <c r="F9" t="s">
-        <v>23</v>
-      </c>
-      <c r="G9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>38003781</v>
       </c>
       <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
         <v>24</v>
       </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
       <c r="D10">
         <v>0</v>
       </c>
-      <c r="E10" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>38004154</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
+        <v>26.74540816326531</v>
+      </c>
+      <c r="G11" t="s">
         <v>26</v>
       </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11" s="2">
-        <v>26.74540816326531</v>
-      </c>
-      <c r="F11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>38003731</v>
       </c>
       <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" t="s">
         <v>28</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2">
+        <v>31.72</v>
+      </c>
+      <c r="G12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" t="s">
         <v>29</v>
       </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12" s="2">
-        <v>31.72</v>
-      </c>
-      <c r="F12" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>38004445</v>
       </c>
       <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" t="s">
         <v>31</v>
       </c>
-      <c r="C13" t="s">
-        <v>32</v>
-      </c>
       <c r="D13">
         <v>0</v>
       </c>
-      <c r="E13" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>38004512</v>
       </c>
       <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
         <v>33</v>
       </c>
-      <c r="C14" t="s">
-        <v>34</v>
-      </c>
       <c r="D14">
         <v>0</v>
       </c>
-      <c r="E14" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>38004446</v>
       </c>
       <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
         <v>35</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15" s="2">
+        <v>42</v>
+      </c>
+      <c r="G15" t="s">
         <v>36</v>
       </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-      <c r="E15" s="2">
-        <v>42</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="H15" t="s">
         <v>37</v>
       </c>
-      <c r="G15" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>38003638</v>
       </c>
       <c r="B16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" t="s">
         <v>39</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16" s="2">
+        <v>71.5</v>
+      </c>
+      <c r="G16" t="s">
         <v>40</v>
       </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16" s="2">
-        <v>71.5</v>
-      </c>
-      <c r="F16" t="s">
-        <v>41</v>
-      </c>
-      <c r="G16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>38003794</v>
       </c>
       <c r="B17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" t="s">
         <v>42</v>
       </c>
-      <c r="C17" t="s">
-        <v>43</v>
-      </c>
       <c r="D17">
         <v>1</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2">
         <v>31.72</v>
       </c>
-      <c r="F17" t="s">
-        <v>23</v>
-      </c>
       <c r="G17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="H17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>38004371</v>
       </c>
       <c r="B18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" t="s">
         <v>44</v>
       </c>
-      <c r="C18" t="s">
-        <v>45</v>
-      </c>
       <c r="D18">
         <v>0</v>
       </c>
-      <c r="E18" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>38004499</v>
       </c>
       <c r="B19" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2">
+        <v>44</v>
+      </c>
+      <c r="G19" t="s">
         <v>46</v>
       </c>
-      <c r="C19" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19">
-        <v>1</v>
-      </c>
-      <c r="E19" s="2">
-        <v>44</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="H19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>0</v>
+      </c>
+      <c r="B20" t="s">
         <v>47</v>
       </c>
-      <c r="G19" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>0</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>48</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20" s="2">
+        <v>42</v>
+      </c>
+      <c r="G20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H20" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>0</v>
+      </c>
+      <c r="B21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" t="s">
         <v>49</v>
       </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20" s="2">
-        <v>42</v>
-      </c>
-      <c r="F20" t="s">
-        <v>37</v>
-      </c>
-      <c r="G20" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>0</v>
-      </c>
-      <c r="B21" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" t="s">
-        <v>50</v>
-      </c>
       <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21" s="2">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21" s="2">
         <v>71.5</v>
       </c>
-      <c r="F21" t="s">
-        <v>41</v>
-      </c>
       <c r="G21" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="H21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>38003625</v>
       </c>
       <c r="B22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s">
         <v>51</v>
       </c>
-      <c r="C22" t="s">
-        <v>52</v>
-      </c>
       <c r="D22">
         <v>0</v>
       </c>
-      <c r="E22" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>38003819</v>
       </c>
       <c r="B23" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" t="s">
         <v>53</v>
       </c>
-      <c r="C23" t="s">
-        <v>54</v>
-      </c>
       <c r="D23">
         <v>0</v>
       </c>
-      <c r="E23" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>38004185</v>
       </c>
       <c r="B24" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D24">
         <v>0</v>
       </c>
-      <c r="E24" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>38004154</v>
       </c>
       <c r="B25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D25">
         <v>0</v>
       </c>
-      <c r="E25" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>38004153</v>
       </c>
       <c r="B26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" t="s">
         <v>57</v>
       </c>
-      <c r="C26" t="s">
-        <v>58</v>
-      </c>
       <c r="D26">
         <v>0</v>
       </c>
-      <c r="E26" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>38003794</v>
       </c>
       <c r="B27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D27">
         <v>1</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27" s="2">
         <v>26.74540816326531</v>
       </c>
-      <c r="F27" t="s">
-        <v>27</v>
-      </c>
       <c r="G27" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="H27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>38004487</v>
       </c>
       <c r="B28" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" t="s">
         <v>60</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2">
+        <v>19.196153846153848</v>
+      </c>
+      <c r="G28" t="s">
         <v>61</v>
       </c>
-      <c r="D28">
-        <v>1</v>
-      </c>
-      <c r="E28" s="2">
-        <v>19.196153846153848</v>
-      </c>
-      <c r="F28" t="s">
-        <v>62</v>
-      </c>
-      <c r="G28" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H28" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>38004185</v>
       </c>
       <c r="B29" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D29">
         <v>0</v>
       </c>
-      <c r="E29" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>38004176</v>
       </c>
       <c r="B30" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" t="s">
         <v>64</v>
       </c>
-      <c r="C30" t="s">
-        <v>65</v>
-      </c>
       <c r="D30">
         <v>0</v>
       </c>
-      <c r="E30" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>38003696</v>
       </c>
       <c r="B31" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C31" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31">
+        <v>1</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31" s="2">
+        <v>28.5</v>
+      </c>
+      <c r="G31" t="s">
         <v>66</v>
       </c>
-      <c r="D31">
-        <v>1</v>
-      </c>
-      <c r="E31" s="2">
-        <v>28.5</v>
-      </c>
-      <c r="F31" t="s">
-        <v>67</v>
-      </c>
-      <c r="G31" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H31" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>38003659</v>
       </c>
       <c r="B32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" t="s">
         <v>68</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32" s="2">
+        <v>53</v>
+      </c>
+      <c r="G32" t="s">
         <v>69</v>
       </c>
-      <c r="D32">
-        <v>1</v>
-      </c>
-      <c r="E32" s="2">
-        <v>53</v>
-      </c>
-      <c r="F32" t="s">
-        <v>70</v>
-      </c>
-      <c r="G32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>38004145</v>
       </c>
       <c r="B33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D33">
         <v>0</v>
       </c>
-      <c r="E33" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E33">
+        <v>0</v>
+      </c>
+      <c r="F33" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>38003731</v>
       </c>
       <c r="B34" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C34" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D34">
         <v>0</v>
       </c>
-      <c r="E34" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>38004512</v>
       </c>
       <c r="B35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C35" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D35">
         <v>0</v>
       </c>
-      <c r="E35" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>38004169</v>
       </c>
       <c r="B36" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" t="s">
         <v>74</v>
       </c>
-      <c r="C36" t="s">
-        <v>75</v>
-      </c>
       <c r="D36">
         <v>0</v>
       </c>
-      <c r="E36" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>38003789</v>
       </c>
       <c r="B37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C37" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D37">
         <v>0</v>
       </c>
-      <c r="E37" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>38003716</v>
       </c>
       <c r="B38" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" t="s">
         <v>77</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38" s="2">
+        <v>42</v>
+      </c>
+      <c r="G38" t="s">
         <v>78</v>
       </c>
-      <c r="D38">
-        <v>1</v>
-      </c>
-      <c r="E38" s="2">
-        <v>42</v>
-      </c>
-      <c r="F38" t="s">
-        <v>79</v>
-      </c>
-      <c r="G38" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H38" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38004390</v>
       </c>
       <c r="B39" t="s">
+        <v>79</v>
+      </c>
+      <c r="C39" t="s">
         <v>80</v>
       </c>
-      <c r="C39" t="s">
-        <v>81</v>
-      </c>
       <c r="D39">
         <v>1</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39" s="2">
         <v>26.74540816326531</v>
       </c>
-      <c r="F39" t="s">
-        <v>27</v>
-      </c>
       <c r="G39" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="H39" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>38004446</v>
       </c>
       <c r="B40" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C40" t="s">
+        <v>81</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40" s="2">
+        <v>42</v>
+      </c>
+      <c r="G40" t="s">
+        <v>36</v>
+      </c>
+      <c r="H40" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>0</v>
+      </c>
+      <c r="B41" t="s">
+        <v>47</v>
+      </c>
+      <c r="C41" t="s">
         <v>82</v>
       </c>
-      <c r="D40">
-        <v>1</v>
-      </c>
-      <c r="E40" s="2">
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41" s="2">
         <v>42</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G41" t="s">
+        <v>36</v>
+      </c>
+      <c r="H41" t="s">
         <v>37</v>
       </c>
-      <c r="G40" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>0</v>
-      </c>
-      <c r="B41" t="s">
-        <v>48</v>
-      </c>
-      <c r="C41" t="s">
-        <v>83</v>
-      </c>
-      <c r="D41">
-        <v>1</v>
-      </c>
-      <c r="E41" s="2">
-        <v>42</v>
-      </c>
-      <c r="F41" t="s">
-        <v>37</v>
-      </c>
-      <c r="G41" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>38003690</v>
       </c>
       <c r="B42" t="s">
+        <v>83</v>
+      </c>
+      <c r="C42" t="s">
         <v>84</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42" s="2">
+        <v>39</v>
+      </c>
+      <c r="G42" t="s">
         <v>85</v>
       </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
-      <c r="E42" s="2">
-        <v>39</v>
-      </c>
-      <c r="F42" t="s">
-        <v>86</v>
-      </c>
-      <c r="G42" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H42" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>38004185</v>
       </c>
       <c r="B43" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C43" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D43">
         <v>0</v>
       </c>
-      <c r="E43" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>38004154</v>
       </c>
       <c r="B44" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C44" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>0</v>
+      </c>
+      <c r="B45" t="s">
+        <v>47</v>
+      </c>
+      <c r="C45" t="s">
         <v>88</v>
       </c>
-      <c r="D44">
-        <v>0</v>
-      </c>
-      <c r="E44" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>0</v>
-      </c>
-      <c r="B45" t="s">
-        <v>48</v>
-      </c>
-      <c r="C45" t="s">
-        <v>89</v>
-      </c>
       <c r="D45">
-        <v>1</v>
-      </c>
-      <c r="E45" s="2">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
+      <c r="F45" s="2">
         <v>42</v>
       </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
+        <v>36</v>
+      </c>
+      <c r="H45" t="s">
         <v>37</v>
       </c>
-      <c r="G45" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>38003794</v>
       </c>
       <c r="B46" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D46">
         <v>1</v>
       </c>
-      <c r="E46" s="2">
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46" s="2">
         <v>31.72</v>
       </c>
-      <c r="F46" t="s">
-        <v>23</v>
-      </c>
       <c r="G46" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="H46" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>38004370</v>
       </c>
       <c r="B47" t="s">
+        <v>90</v>
+      </c>
+      <c r="C47" t="s">
         <v>91</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47" s="2">
+        <v>19.196153846153848</v>
+      </c>
+      <c r="G47" t="s">
         <v>92</v>
       </c>
-      <c r="D47">
-        <v>1</v>
-      </c>
-      <c r="E47" s="2">
-        <v>19.196153846153848</v>
-      </c>
-      <c r="F47" t="s">
-        <v>93</v>
-      </c>
-      <c r="G47" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H47" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>38004056</v>
       </c>
       <c r="B48" t="s">
+        <v>93</v>
+      </c>
+      <c r="C48" t="s">
         <v>94</v>
       </c>
-      <c r="C48" t="s">
-        <v>95</v>
-      </c>
       <c r="D48">
         <v>1</v>
       </c>
-      <c r="E48" s="2">
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48" s="2">
         <v>41</v>
       </c>
-      <c r="F48" t="s">
-        <v>17</v>
-      </c>
       <c r="G48" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="H48" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>38003781</v>
       </c>
       <c r="B49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C49" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D49">
         <v>0</v>
       </c>
-      <c r="E49" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E49">
+        <v>0</v>
+      </c>
+      <c r="F49" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>38003819</v>
       </c>
       <c r="B50" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C50" t="s">
+        <v>96</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+      <c r="F50" s="2">
+        <v>6</v>
+      </c>
+      <c r="G50" t="s">
         <v>97</v>
       </c>
-      <c r="D50">
-        <v>1</v>
-      </c>
-      <c r="E50" s="2">
-        <v>6</v>
-      </c>
-      <c r="F50" t="s">
-        <v>98</v>
-      </c>
-      <c r="G50" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H50" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>38003731</v>
       </c>
       <c r="B51" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C51" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D51">
         <v>1</v>
       </c>
-      <c r="E51" s="2">
+      <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="F51" s="2">
         <v>42</v>
       </c>
-      <c r="F51" t="s">
-        <v>79</v>
-      </c>
       <c r="G51" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="H51" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>38004512</v>
       </c>
       <c r="B52" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C52" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D52">
         <v>0</v>
       </c>
-      <c r="E52" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>38003722</v>
       </c>
       <c r="B53" t="s">
+        <v>99</v>
+      </c>
+      <c r="C53" t="s">
         <v>100</v>
       </c>
-      <c r="C53" t="s">
-        <v>101</v>
-      </c>
       <c r="D53">
         <v>1</v>
       </c>
-      <c r="E53" s="2">
+      <c r="E53">
+        <v>1</v>
+      </c>
+      <c r="F53" s="2">
         <v>19.196153846153848</v>
       </c>
-      <c r="F53" t="s">
-        <v>62</v>
-      </c>
       <c r="G53" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="H53" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>38004030</v>
       </c>
       <c r="B54" t="s">
+        <v>101</v>
+      </c>
+      <c r="C54" t="s">
         <v>102</v>
       </c>
-      <c r="C54" t="s">
-        <v>103</v>
-      </c>
       <c r="D54">
         <v>1</v>
       </c>
-      <c r="E54" s="2">
+      <c r="E54">
+        <v>1</v>
+      </c>
+      <c r="F54" s="2">
         <v>41</v>
       </c>
-      <c r="F54" t="s">
-        <v>17</v>
-      </c>
       <c r="G54" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="H54" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>38004413</v>
       </c>
       <c r="B55" t="s">
+        <v>103</v>
+      </c>
+      <c r="C55" t="s">
         <v>104</v>
       </c>
-      <c r="C55" t="s">
-        <v>105</v>
-      </c>
       <c r="D55">
         <v>1</v>
       </c>
-      <c r="E55" s="2">
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55" s="2">
         <v>26.74540816326531</v>
       </c>
-      <c r="F55" t="s">
-        <v>27</v>
-      </c>
       <c r="G55" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="H55" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>38004185</v>
       </c>
       <c r="B56" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C56" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D56">
         <v>0</v>
       </c>
-      <c r="E56" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>38004169</v>
       </c>
       <c r="B57" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C57" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D57">
         <v>0</v>
       </c>
-      <c r="E57" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>38003760</v>
       </c>
       <c r="B58" t="s">
+        <v>107</v>
+      </c>
+      <c r="C58" t="s">
         <v>108</v>
       </c>
-      <c r="C58" t="s">
-        <v>109</v>
-      </c>
       <c r="D58">
         <v>1</v>
       </c>
-      <c r="E58" s="2">
+      <c r="E58">
+        <v>1</v>
+      </c>
+      <c r="F58" s="2">
         <v>19.196153846153848</v>
       </c>
-      <c r="F58" t="s">
-        <v>62</v>
-      </c>
       <c r="G58" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="H58" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>38003807</v>
       </c>
       <c r="B59" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C59" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D59">
         <v>1</v>
       </c>
-      <c r="E59" s="2">
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="F59" s="2">
         <v>31.72</v>
       </c>
-      <c r="F59" t="s">
-        <v>23</v>
-      </c>
       <c r="G59" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="H59" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>38004154</v>
       </c>
       <c r="B60" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C60" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D60">
         <v>0</v>
       </c>
-      <c r="E60" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>38003716</v>
       </c>
       <c r="B61" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C61" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D61">
         <v>1</v>
       </c>
-      <c r="E61" s="2">
+      <c r="E61">
+        <v>1</v>
+      </c>
+      <c r="F61" s="2">
         <v>42</v>
       </c>
-      <c r="F61" t="s">
-        <v>79</v>
-      </c>
       <c r="G61" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="H61" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>38004376</v>
       </c>
       <c r="B62" t="s">
+        <v>112</v>
+      </c>
+      <c r="C62" t="s">
         <v>113</v>
       </c>
-      <c r="C62" t="s">
-        <v>114</v>
-      </c>
       <c r="D62">
         <v>1</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62">
+        <v>1</v>
+      </c>
+      <c r="F62" s="2">
         <v>42</v>
       </c>
-      <c r="F62" t="s">
+      <c r="G62" t="s">
+        <v>36</v>
+      </c>
+      <c r="H62" t="s">
         <v>37</v>
       </c>
-      <c r="G62" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>38004512</v>
       </c>
       <c r="B63" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C63" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D63">
         <v>1</v>
       </c>
-      <c r="E63" s="2">
+      <c r="E63">
+        <v>1</v>
+      </c>
+      <c r="F63" s="2">
         <v>42</v>
       </c>
-      <c r="F63" t="s">
+      <c r="G63" t="s">
+        <v>36</v>
+      </c>
+      <c r="H63" t="s">
         <v>37</v>
       </c>
-      <c r="G63" t="s">
-        <v>38</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G63" xr:uid="{B01908DF-AC8E-4A47-8381-A0A0F45C789A}"/>
+  <autoFilter ref="A1:H63" xr:uid="{B01908DF-AC8E-4A47-8381-A0A0F45C789A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix to standard omop code to include uncategorised specialties
</commit_message>
<xml_diff>
--- a/provider_specialty_cprd_V.0.4.xlsx
+++ b/provider_specialty_cprd_V.0.4.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioxfordnexus-my.sharepoint.com/personal/orms0952_ox_ac_uk/Documents/OMOP_Validation study/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{03CD51DF-2ED6-4E6D-9395-4CAD2A3CE9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B198807-D701-4EAC-AD25-C244C2969FF4}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="8_{03CD51DF-2ED6-4E6D-9395-4CAD2A3CE9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F87D4C9C-FCA9-438F-99A6-A1932C9E8BE9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{46870897-BCFD-414C-A471-BD3159C3E0A3}"/>
+    <workbookView minimized="1" xWindow="30660" yWindow="1860" windowWidth="18900" windowHeight="10965" xr2:uid="{46870897-BCFD-414C-A471-BD3159C3E0A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$63</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="119">
   <si>
     <t>specialty_concept_id</t>
   </si>
@@ -390,6 +390,12 @@
   </si>
   <si>
     <t>Include_standard</t>
+  </si>
+  <si>
+    <t>specialty_concept_summarised</t>
+  </si>
+  <si>
+    <t>Uncategorised</t>
   </si>
 </sst>
 </file>
@@ -773,7 +779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01908DF-AC8E-4A47-8381-A0A0F45C789A}">
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" bestFit="1" customWidth="1"/>
@@ -782,11 +788,11 @@
     <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="255.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="39.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" customWidth="1"/>
+    <col min="8" max="8" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -811,8 +817,11 @@
       <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>38004185</v>
       </c>
@@ -832,7 +841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>38003696</v>
       </c>
@@ -857,8 +866,11 @@
       <c r="H3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>38004185</v>
       </c>
@@ -878,7 +890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>38004154</v>
       </c>
@@ -898,7 +910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>38003627</v>
       </c>
@@ -923,8 +935,11 @@
       <c r="H6" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>38003810</v>
       </c>
@@ -944,7 +959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>38003648</v>
       </c>
@@ -964,7 +979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>38003789</v>
       </c>
@@ -989,8 +1004,11 @@
       <c r="H9" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>38003781</v>
       </c>
@@ -1010,7 +1028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>38004154</v>
       </c>
@@ -1027,13 +1045,10 @@
         <v>0</v>
       </c>
       <c r="F11" s="2">
-        <v>26.74540816326531</v>
-      </c>
-      <c r="G11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>38003731</v>
       </c>
@@ -1058,8 +1073,11 @@
       <c r="H12" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>38004445</v>
       </c>
@@ -1079,7 +1097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>38004512</v>
       </c>
@@ -1099,7 +1117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>38004446</v>
       </c>
@@ -1124,8 +1142,11 @@
       <c r="H15" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>38003638</v>
       </c>
@@ -1150,8 +1171,11 @@
       <c r="H16" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>38003794</v>
       </c>
@@ -1176,8 +1200,11 @@
       <c r="H17" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>38004371</v>
       </c>
@@ -1197,7 +1224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>38004499</v>
       </c>
@@ -1222,8 +1249,11 @@
       <c r="H19" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>0</v>
       </c>
@@ -1234,7 +1264,7 @@
         <v>48</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -1248,8 +1278,11 @@
       <c r="H20" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I20" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>0</v>
       </c>
@@ -1260,7 +1293,7 @@
         <v>49</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -1274,8 +1307,11 @@
       <c r="H21" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I21" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>38003625</v>
       </c>
@@ -1295,7 +1331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>38003819</v>
       </c>
@@ -1315,7 +1351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>38004185</v>
       </c>
@@ -1335,7 +1371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>38004154</v>
       </c>
@@ -1355,7 +1391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>38004153</v>
       </c>
@@ -1375,7 +1411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>38003794</v>
       </c>
@@ -1400,8 +1436,11 @@
       <c r="H27" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>38004487</v>
       </c>
@@ -1426,8 +1465,11 @@
       <c r="H28" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I28" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>38004185</v>
       </c>
@@ -1447,7 +1489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>38004176</v>
       </c>
@@ -1467,7 +1509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>38003696</v>
       </c>
@@ -1492,8 +1534,11 @@
       <c r="H31" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I31" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>38003659</v>
       </c>
@@ -1518,8 +1563,11 @@
       <c r="H32" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>38004145</v>
       </c>
@@ -1539,7 +1587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>38003731</v>
       </c>
@@ -1559,7 +1607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>38004512</v>
       </c>
@@ -1579,7 +1627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>38004169</v>
       </c>
@@ -1599,7 +1647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>38003789</v>
       </c>
@@ -1619,7 +1667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>38003716</v>
       </c>
@@ -1644,8 +1692,11 @@
       <c r="H38" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I38" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38004390</v>
       </c>
@@ -1670,8 +1721,11 @@
       <c r="H39" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I39" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>38004446</v>
       </c>
@@ -1696,8 +1750,11 @@
       <c r="H40" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I40" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>0</v>
       </c>
@@ -1708,7 +1765,7 @@
         <v>82</v>
       </c>
       <c r="D41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41">
         <v>1</v>
@@ -1722,8 +1779,11 @@
       <c r="H41" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I41" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>38003690</v>
       </c>
@@ -1748,8 +1808,11 @@
       <c r="H42" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I42" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>38004185</v>
       </c>
@@ -1769,7 +1832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>38004154</v>
       </c>
@@ -1789,7 +1852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>0</v>
       </c>
@@ -1800,7 +1863,7 @@
         <v>88</v>
       </c>
       <c r="D45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45">
         <v>1</v>
@@ -1814,8 +1877,11 @@
       <c r="H45" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I45" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>38003794</v>
       </c>
@@ -1840,8 +1906,11 @@
       <c r="H46" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I46" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>38004370</v>
       </c>
@@ -1866,8 +1935,11 @@
       <c r="H47" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I47" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>38004056</v>
       </c>
@@ -1892,8 +1964,11 @@
       <c r="H48" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I48" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>38003781</v>
       </c>
@@ -1913,7 +1988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>38003819</v>
       </c>
@@ -1938,8 +2013,11 @@
       <c r="H50" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I50" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>38003731</v>
       </c>
@@ -1964,8 +2042,11 @@
       <c r="H51" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I51" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>38004512</v>
       </c>
@@ -1985,7 +2066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>38003722</v>
       </c>
@@ -2010,8 +2091,11 @@
       <c r="H53" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I53" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>38004030</v>
       </c>
@@ -2036,8 +2120,11 @@
       <c r="H54" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I54" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>38004413</v>
       </c>
@@ -2062,8 +2149,11 @@
       <c r="H55" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I55" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>38004185</v>
       </c>
@@ -2083,7 +2173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>38004169</v>
       </c>
@@ -2103,7 +2193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>38003760</v>
       </c>
@@ -2128,8 +2218,11 @@
       <c r="H58" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I58" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>38003807</v>
       </c>
@@ -2154,8 +2247,11 @@
       <c r="H59" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I59" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>38004154</v>
       </c>
@@ -2175,7 +2271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>38003716</v>
       </c>
@@ -2200,8 +2296,11 @@
       <c r="H61" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I61" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>38004376</v>
       </c>
@@ -2226,8 +2325,11 @@
       <c r="H62" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I62" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>38004512</v>
       </c>
@@ -2252,9 +2354,12 @@
       <c r="H63" t="s">
         <v>37</v>
       </c>
+      <c r="I63" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H63" xr:uid="{B01908DF-AC8E-4A47-8381-A0A0F45C789A}"/>
+  <autoFilter ref="A1:I63" xr:uid="{B01908DF-AC8E-4A47-8381-A0A0F45C789A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>